<commit_message>
feat: write manifest envelope
</commit_message>
<xml_diff>
--- a/ThunderbirdsBoardGameEngine.Catalog.Generator/Resources/DisasterCards.xlsx
+++ b/ThunderbirdsBoardGameEngine.Catalog.Generator/Resources/DisasterCards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine.GameData.Api\ThunderbirdsBoardGameEngine.GameData.Importer\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\ThunderbirdsBoardGameEngine.Catalog.Generator\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF60A780-F584-46F3-BC31-222A55F7637C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E467C19-7FA8-41B2-A114-7B2F220524AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
@@ -239,9 +239,6 @@
     <t>Alan</t>
   </si>
   <si>
-    <t>Attack of the Aligators</t>
-  </si>
-  <si>
     <t>Atlantic Inferno</t>
   </si>
   <si>
@@ -323,10 +320,13 @@
     <t>Martian Invasion</t>
   </si>
   <si>
-    <t>Day of Disater</t>
-  </si>
-  <si>
     <t>They Call Him Mr. X</t>
+  </si>
+  <si>
+    <t>Attack of the Alligators</t>
+  </si>
+  <si>
+    <t>Day of Disaster</t>
   </si>
 </sst>
 </file>
@@ -1251,7 +1251,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="B17">
         <v>10</v>
@@ -1283,13 +1283,13 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B18">
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
@@ -1315,7 +1315,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -1327,7 +1327,7 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19">
         <v>3</v>
@@ -1344,7 +1344,7 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20">
         <v>11</v>
@@ -1382,13 +1382,13 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21">
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D21" t="s">
         <v>17</v>
@@ -1412,7 +1412,7 @@
         <v>2</v>
       </c>
       <c r="M21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N21" t="s">
         <v>27</v>
@@ -1423,13 +1423,13 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D22" t="s">
         <v>17</v>
@@ -1455,13 +1455,13 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23">
         <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -1484,13 +1484,13 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B24">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
@@ -1519,7 +1519,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25">
         <v>8</v>
@@ -1548,7 +1548,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26">
         <v>8</v>
@@ -1560,7 +1560,7 @@
         <v>48</v>
       </c>
       <c r="E26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F26">
         <v>3</v>
@@ -1577,13 +1577,13 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
         <v>37</v>
@@ -1601,7 +1601,7 @@
         <v>2</v>
       </c>
       <c r="J27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N27" t="s">
         <v>27</v>
@@ -1612,7 +1612,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -1624,7 +1624,7 @@
         <v>24</v>
       </c>
       <c r="E28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F28">
         <v>3</v>
@@ -1647,13 +1647,13 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B29">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D29" t="s">
         <v>48</v>
@@ -1682,13 +1682,13 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30">
         <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D30" t="s">
         <v>48</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B31">
         <v>7</v>
@@ -1738,7 +1738,7 @@
         <v>2</v>
       </c>
       <c r="J31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N31" t="s">
         <v>27</v>
@@ -1746,13 +1746,13 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B32">
         <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B33">
         <v>7</v>
@@ -1798,7 +1798,7 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B34">
         <v>9</v>
@@ -1830,7 +1830,7 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B35">
         <v>8</v>
@@ -1842,19 +1842,19 @@
         <v>48</v>
       </c>
       <c r="E35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="H35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I35">
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L35">
         <v>2</v>

</xml_diff>